<commit_message>
feat(dcm): J02 gen_dcm_arxml 新增 DcmDspSession/DcmDspSecurity 容器重建
- Parse_dcm_dsp_excel: 解析问卷 DcmDspSession/DcmDspSecurity 表 (空属性不生成)
- Rebuild_DcmDsp: 定位两容器清空 SUB-CONTAINERS 并按 Excel 重建,
  参数顺序/元素类型对齐基线 arxml, 容器级参数与兄弟容器逐字节保留
- Dcm_arxml_Script: 接线 + DcmDspSessionRow/DcmDspSecurityRow 锚点兜底
- 问卷模板补充 DcmDspSession/DcmDspSecurity 两 sheet

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/UDS_Diagnostic_Questionnaire/UDS_Diagnostic_Questionnaire_Template.xlsx
+++ b/UDS_Diagnostic_Questionnaire/UDS_Diagnostic_Questionnaire_Template.xlsx
@@ -12,6 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DID List" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RID List" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NVM List" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DcmDspSecurity" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DcmDspSession" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'History'!$A$2:$E$32</definedName>
@@ -20,6 +22,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'DID List'!$A$2:$Q$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'RID List'!$A$2:$P$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'NVM List'!$A$2:$K$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'DcmDspSecurity'!$A$1:$Q$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'DcmDspSession'!$A$1:$E$4</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -4952,4 +4956,408 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="31" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="27" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="36" customWidth="1" min="13" max="13"/>
+    <col width="23" customWidth="1" min="14" max="14"/>
+    <col width="28" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="16" max="16"/>
+    <col width="36" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>DcmDspSecurityRow</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>DcmDspSecurityADRSize</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>DcmDspSecurityAttemptCounterEnabled</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>DcmDspSecurityCompareKeyFnc</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>DcmDspSecurityDelayTime</t>
+        </is>
+      </c>
+      <c r="F1" s="11" t="inlineStr">
+        <is>
+          <t>DcmDspSecurityDelayTimeOnBoot</t>
+        </is>
+      </c>
+      <c r="G1" s="11" t="inlineStr">
+        <is>
+          <t>DcmDspSecurityGetAttemptCounterFnc</t>
+        </is>
+      </c>
+      <c r="H1" s="11" t="inlineStr">
+        <is>
+          <t>DcmDspSecurityGetSeedFnc</t>
+        </is>
+      </c>
+      <c r="I1" s="11" t="inlineStr">
+        <is>
+          <t>DcmDspSecurityKeySize</t>
+        </is>
+      </c>
+      <c r="J1" s="11" t="inlineStr">
+        <is>
+          <t>DcmDspSecurityLevel</t>
+        </is>
+      </c>
+      <c r="K1" s="11" t="inlineStr">
+        <is>
+          <t>DcmDspSecurityNumAttDelay</t>
+        </is>
+      </c>
+      <c r="L1" s="11" t="inlineStr">
+        <is>
+          <t>DcmDspSecuritySeedSize</t>
+        </is>
+      </c>
+      <c r="M1" s="11" t="inlineStr">
+        <is>
+          <t>DcmDspSecuritySetAttemptCounterFnc</t>
+        </is>
+      </c>
+      <c r="N1" s="11" t="inlineStr">
+        <is>
+          <t>DcmDspSecurityUsePort</t>
+        </is>
+      </c>
+      <c r="O1" s="11" t="inlineStr">
+        <is>
+          <t>DcmRbDspSecurityNumAttLock</t>
+        </is>
+      </c>
+      <c r="P1" s="11" t="inlineStr">
+        <is>
+          <t>DcmRbDspSecurityRowUseAsynchronousServerCallPoint</t>
+        </is>
+      </c>
+      <c r="Q1" s="11" t="inlineStr">
+        <is>
+          <t>DcmRbDspSecurityRowUseFlexibleLength</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>Unlocked_L3</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="n"/>
+      <c r="C2" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D2" s="13" t="inlineStr">
+        <is>
+          <t>BootSecurityCompareKey</t>
+        </is>
+      </c>
+      <c r="E2" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="F2" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="G2" s="13" t="inlineStr">
+        <is>
+          <t>BootSecurityGetAttempCount</t>
+        </is>
+      </c>
+      <c r="H2" s="13" t="inlineStr">
+        <is>
+          <t>BootSecurityGetSeed</t>
+        </is>
+      </c>
+      <c r="I2" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="J2" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="K2" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="L2" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="M2" s="13" t="inlineStr">
+        <is>
+          <t>BootSecuritySetAttempCount</t>
+        </is>
+      </c>
+      <c r="N2" s="13" t="inlineStr">
+        <is>
+          <t>USE_ASYNCH_FNC</t>
+        </is>
+      </c>
+      <c r="O2" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" s="13" t="n"/>
+      <c r="Q2" s="13" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>Unlocked_L1</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="n"/>
+      <c r="C3" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>AppSecurityCompareKey</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="F3" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>AppSecurityGetAttempCount</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>AppSecurityGetSeed</t>
+        </is>
+      </c>
+      <c r="I3" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="J3" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="L3" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="M3" s="13" t="inlineStr">
+        <is>
+          <t>AppSecuritySetAttempCount</t>
+        </is>
+      </c>
+      <c r="N3" s="13" t="inlineStr">
+        <is>
+          <t>USE_ASYNCH_FNC</t>
+        </is>
+      </c>
+      <c r="O3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" s="13" t="n"/>
+      <c r="Q3" s="13" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Unlocked_L49</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="n">
+        <v>16</v>
+      </c>
+      <c r="C4" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>DevelopSecurityCompareKey</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="F4" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="G4" s="13" t="n"/>
+      <c r="H4" s="13" t="inlineStr">
+        <is>
+          <t>DevelopSecurityGetSeed</t>
+        </is>
+      </c>
+      <c r="I4" s="13" t="n">
+        <v>16</v>
+      </c>
+      <c r="J4" s="13" t="n">
+        <v>49</v>
+      </c>
+      <c r="K4" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="L4" s="13" t="n">
+        <v>16</v>
+      </c>
+      <c r="M4" s="13" t="n"/>
+      <c r="N4" s="13" t="inlineStr">
+        <is>
+          <t>USE_ASYNCH_FNC</t>
+        </is>
+      </c>
+      <c r="O4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" s="13" t="n"/>
+      <c r="Q4" s="13" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:Q4"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>DcmDspSessionRow</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>DcmDspSessionForBoot</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>DcmDspSessionLevel</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>DcmDspSessionP2ServerMax</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>DcmDspSessionP2StarServerMax</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>DEFAULT_SESSION</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>DCM_NO_BOOT</t>
+        </is>
+      </c>
+      <c r="C2" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E2" s="13" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>PROGRAMMING_SESSION</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>DCM_NO_BOOT</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E3" s="13" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>EXTENDED_DIAGNOSTIC_SESSION</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>DCM_NO_BOOT</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E4" s="13" t="n">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E4"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(dcm): J02 DcmDspSecurity 行更名 Unlocked_L1/L3/L49 -> Unlocked_App/Boot/Develop
- Excel (J02 + 模板) DcmDspSecurity sheet 行名同步 (zip 级替换, 仅动行名字符串)
- Create_DcmDsdServices SECURITY_MAP 引用目标同步,
  服务表 DcmDsdSidTabSecurityLevelRef 随之指向新行名
- J02 安全行配置更新 (Level/KeySize/SeedSize/AttemptCounter, 含 App Level=2
  适配 SecurityAccess 子 ID 0x3/0x4 匹配规则)

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/UDS_Diagnostic_Questionnaire/UDS_Diagnostic_Questionnaire_Template.xlsx
+++ b/UDS_Diagnostic_Questionnaire/UDS_Diagnostic_Questionnaire_Template.xlsx
@@ -5076,7 +5076,7 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>Unlocked_L3</t>
+          <t>Unlocked_Boot</t>
         </is>
       </c>
       <c r="B2" s="13" t="n"/>
@@ -5135,7 +5135,7 @@
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>Unlocked_L1</t>
+          <t>Unlocked_App</t>
         </is>
       </c>
       <c r="B3" s="13" t="n"/>
@@ -5194,7 +5194,7 @@
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
-          <t>Unlocked_L49</t>
+          <t>Unlocked_Develop</t>
         </is>
       </c>
       <c r="B4" s="13" t="n">

</xml_diff>